<commit_message>
Updated Zergaw_territory_transaction_chart with updated work
</commit_message>
<xml_diff>
--- a/Zergaw_territory_transaction_chart.xlsx
+++ b/Zergaw_territory_transaction_chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tihitinazergaw\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F551B72F-F3E2-45BD-825E-814F7F6471FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F41C81C-5C40-4AF8-8F6E-405773A5864C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E2915678-4855-4884-8A79-49E8D6774CEB}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="6" r:id="rId2"/>
+    <pivotCache cacheId="1" r:id="rId2"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -542,9 +542,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -915,6 +914,9 @@
       <c:pivotFmt>
         <c:idx val="4"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -1027,6 +1029,9 @@
       <c:pivotFmt>
         <c:idx val="6"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -1083,6 +1088,9 @@
       <c:pivotFmt>
         <c:idx val="7"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -2212,6 +2220,69 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5632450" cy="785260"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7FDC295-42CD-06A9-DE60-952D487B4871}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4267200" y="7550150"/>
+          <a:ext cx="5632450" cy="785260"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>This chart</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> compares the number of transactions and average transaction size in 2025. While October has the highst number of transaction, August stands out because both number of transactions and average transaction size are high, which explains why August has the highest revenue.</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4334,7 +4405,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8B7DAB40-34F4-4103-9040-DE0F34FE5774}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8B7DAB40-34F4-4103-9040-DE0F34FE5774}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="H3:L18" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisCol" showAll="0">
@@ -5033,7 +5104,7 @@
       <c r="E3">
         <v>21.43</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -5079,7 +5150,7 @@
       <c r="E5">
         <v>46.23</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="I5" t="s">
@@ -5105,19 +5176,19 @@
       <c r="E6">
         <v>8.73</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="2">
         <v>1</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6">
         <v>142</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="3">
         <v>132.37333333333333</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6">
         <v>142</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="3">
         <v>132.37333333333333</v>
       </c>
     </row>
@@ -5137,19 +5208,19 @@
       <c r="E7">
         <v>24.04</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="2">
         <v>2</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7">
         <v>117</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="3">
         <v>114.83666666666666</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7">
         <v>117</v>
       </c>
-      <c r="L7" s="4">
+      <c r="L7" s="3">
         <v>114.83666666666666</v>
       </c>
     </row>
@@ -5169,19 +5240,19 @@
       <c r="E8">
         <v>549.86</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="2">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8">
         <v>137</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="3">
         <v>125.50333333333333</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8">
         <v>137</v>
       </c>
-      <c r="L8" s="4">
+      <c r="L8" s="3">
         <v>125.50333333333333</v>
       </c>
     </row>
@@ -5201,19 +5272,19 @@
       <c r="E9">
         <v>48.04</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="2">
         <v>4</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9">
         <v>171</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="3">
         <v>145.465</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9">
         <v>171</v>
       </c>
-      <c r="L9" s="4">
+      <c r="L9" s="3">
         <v>145.465</v>
       </c>
     </row>
@@ -5233,19 +5304,19 @@
       <c r="E10">
         <v>9.34</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="2">
         <v>5</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10">
         <v>156</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="3">
         <v>125.73333333333335</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10">
         <v>156</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="3">
         <v>125.73333333333335</v>
       </c>
     </row>
@@ -5265,19 +5336,19 @@
       <c r="E11">
         <v>22.96</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="2">
         <v>6</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11">
         <v>144</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="3">
         <v>140.995</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11">
         <v>144</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L11" s="3">
         <v>140.995</v>
       </c>
     </row>
@@ -5297,19 +5368,19 @@
       <c r="E12">
         <v>31.12</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="2">
         <v>7</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12">
         <v>140</v>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="3">
         <v>121.56333333333332</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12">
         <v>140</v>
       </c>
-      <c r="L12" s="4">
+      <c r="L12" s="3">
         <v>121.56333333333332</v>
       </c>
     </row>
@@ -5329,19 +5400,19 @@
       <c r="E13">
         <v>193.67</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="2">
         <v>8</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13">
         <v>166</v>
       </c>
-      <c r="J13" s="4">
+      <c r="J13" s="3">
         <v>160.08500000000001</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13">
         <v>166</v>
       </c>
-      <c r="L13" s="4">
+      <c r="L13" s="3">
         <v>160.08500000000001</v>
       </c>
     </row>
@@ -5361,19 +5432,19 @@
       <c r="E14">
         <v>400.89</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="2">
         <v>9</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14">
         <v>107</v>
       </c>
-      <c r="J14" s="4">
+      <c r="J14" s="3">
         <v>135.57333333333332</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14">
         <v>107</v>
       </c>
-      <c r="L14" s="4">
+      <c r="L14" s="3">
         <v>135.57333333333332</v>
       </c>
     </row>
@@ -5393,19 +5464,19 @@
       <c r="E15">
         <v>23.42</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="2">
         <v>10</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15">
         <v>209</v>
       </c>
-      <c r="J15" s="4">
+      <c r="J15" s="3">
         <v>127.71333333333332</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15">
         <v>209</v>
       </c>
-      <c r="L15" s="4">
+      <c r="L15" s="3">
         <v>127.71333333333332</v>
       </c>
     </row>
@@ -5425,19 +5496,19 @@
       <c r="E16">
         <v>168.55</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="2">
         <v>11</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16">
         <v>119</v>
       </c>
-      <c r="J16" s="4">
+      <c r="J16" s="3">
         <v>125.12166666666667</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16">
         <v>119</v>
       </c>
-      <c r="L16" s="4">
+      <c r="L16" s="3">
         <v>125.12166666666667</v>
       </c>
     </row>
@@ -5457,19 +5528,19 @@
       <c r="E17">
         <v>30.34</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="2">
         <v>12</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17">
         <v>126</v>
       </c>
-      <c r="J17" s="4">
+      <c r="J17" s="3">
         <v>132.69000000000003</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17">
         <v>126</v>
       </c>
-      <c r="L17" s="4">
+      <c r="L17" s="3">
         <v>132.69000000000003</v>
       </c>
     </row>
@@ -5489,19 +5560,19 @@
       <c r="E18">
         <v>8.9700000000000006</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="H18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I18" s="1">
+      <c r="I18">
         <v>1734</v>
       </c>
-      <c r="J18" s="4">
+      <c r="J18" s="3">
         <v>132.3044444444445</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18">
         <v>1734</v>
       </c>
-      <c r="L18" s="4">
+      <c r="L18" s="3">
         <v>132.30444444444441</v>
       </c>
     </row>

</xml_diff>